<commit_message>
modified input file data
</commit_message>
<xml_diff>
--- a/data/WHRS - INPUT FILE.xlsx
+++ b/data/WHRS - INPUT FILE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VENKAT\Downloads\LEARNING\WHRS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFB9AAA-4D86-481A-89A2-5CFA18ED4682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CC206D-308E-455F-8B95-DDE0750CE1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3746,6 +3746,15 @@
       <c r="T42" t="s">
         <v>37</v>
       </c>
+      <c r="U42">
+        <v>60888</v>
+      </c>
+      <c r="V42">
+        <v>63776</v>
+      </c>
+      <c r="W42">
+        <v>0</v>
+      </c>
     </row>
     <row r="43" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A43" s="1">
@@ -3771,6 +3780,15 @@
       </c>
       <c r="T43" t="s">
         <v>37</v>
+      </c>
+      <c r="U43">
+        <v>60888</v>
+      </c>
+      <c r="V43">
+        <v>63776</v>
+      </c>
+      <c r="W43">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>